<commit_message>
Accept Unknown and Non-cape, and tell blanks apart from Unknown
From tester feedback:
- Disposition can now be Unknown or Non-cape; Status (and Gender) can be
  Unknown. The workbook's Lists sheet and Disposition dropdown include the
  new values, and the build accepts them even if a sheet doesn't list them.
  "Noncape"/"non cape" spellings are normalised to Non-cape.
- People marked Non-cape need no power class, are never daily answers, and
  show "No powers" instead of a blank.
- "File incomplete" now means a detail is actually missing, tracked as a
  separate "complete" flag from answer eligibility.
- Blank details read "Not on file" so they can't be confused with a real
  "Unknown" answer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2rJagsxGbYcrTNoNQYqhz
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -14828,6 +14828,9 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>1866</v>
+      </c>
       <c r="B5" s="8" t="s">
         <v>1869</v>
       </c>
@@ -14845,6 +14848,11 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Non-cape</t>
+        </is>
+      </c>
       <c r="B6" s="8" t="s">
         <v>595</v>
       </c>
@@ -51948,7 +51956,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
-            <xm:f>Lists!$A$2:$A$4</xm:f>
+            <xm:f>Lists!$A$2:$A$6</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>
@@ -52053,8 +52061,10 @@
       <c r="B2" s="7" t="s">
         <v>1687</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>1688</v>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Hero / Villain / Rogue / Unknown / Non-cape</t>
+        </is>
       </c>
       <c r="D2" s="7" t="s">
         <v>1689</v>

</xml_diff>

<commit_message>
Updates more A capes
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0CAD6E-C2B5-40D6-9222-4F7948D89EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851A60DF-75E6-4CAD-972E-9026055D9E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6870" yWindow="6705" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9386" uniqueCount="1874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9406" uniqueCount="1874">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -14908,7 +14908,7 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -15206,8 +15206,12 @@
       <c r="F5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>1865</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I5" s="5" t="s">
         <v>71</v>
       </c>
@@ -15225,11 +15229,11 @@
       <c r="O5" s="5"/>
       <c r="P5" s="6">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q5" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R5" s="5" t="s">
         <v>51</v>
@@ -15255,7 +15259,9 @@
       <c r="D6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F6" s="5" t="s">
         <v>46</v>
       </c>
@@ -15282,11 +15288,11 @@
       <c r="O6" s="5"/>
       <c r="P6" s="6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>51</v>
@@ -15517,15 +15523,27 @@
         <v>102</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="C10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H10" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="I10" s="5"/>
+      <c r="I10" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
@@ -15538,11 +15556,11 @@
       </c>
       <c r="P10" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R10" s="5" t="s">
         <v>51</v>
@@ -15721,7 +15739,9 @@
       <c r="G13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I13" s="5" t="s">
         <v>123</v>
       </c>
@@ -15737,11 +15757,11 @@
       <c r="O13" s="5"/>
       <c r="P13" s="6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R13" s="5" t="s">
         <v>125</v>
@@ -15781,7 +15801,9 @@
       <c r="H14" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="I14" s="5"/>
+      <c r="I14" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -15792,11 +15814,11 @@
       <c r="O14" s="5"/>
       <c r="P14" s="6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q14" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R14" s="5" t="s">
         <v>51</v>
@@ -15834,7 +15856,9 @@
       <c r="F15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="G15" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>132</v>
       </c>
@@ -15855,11 +15879,11 @@
       <c r="O15" s="5"/>
       <c r="P15" s="6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q15" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R15" s="5" t="s">
         <v>51</v>
@@ -16011,17 +16035,30 @@
         <v>146</v>
       </c>
       <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="C18" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
+      <c r="I18" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>78</v>
+      </c>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="5" t="s">
@@ -16029,12 +16066,12 @@
       </c>
       <c r="O18" s="5"/>
       <c r="P18" s="6">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IF(A18="","",COUNTA(D18:F18)+COUNTA(G18:G18)+COUNTA(H18:H18)+COUNTA(#REF!))</f>
+        <v>6</v>
       </c>
       <c r="Q18" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R18" s="5" t="s">
         <v>51</v>
@@ -43425,7 +43462,9 @@
       <c r="F504" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G504" s="5"/>
+      <c r="G504" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="H504" s="5" t="s">
         <v>664</v>
       </c>
@@ -43444,11 +43483,11 @@
       <c r="O504" s="5"/>
       <c r="P504" s="6">
         <f t="shared" si="14"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q504" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R504" s="5" t="s">
         <v>51</v>
@@ -52080,11 +52119,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D701)</f>
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E2/COUNTA(Roster!A2:A701))</f>
-        <v>0.53728813559322031</v>
+        <v>0.54067796610169494</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -52102,11 +52141,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E701)</f>
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E3/COUNTA(Roster!A2:A701))</f>
-        <v>0.38474576271186439</v>
+        <v>0.38983050847457629</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52124,11 +52163,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F701)</f>
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E4/COUNTA(Roster!A2:A701))</f>
-        <v>0.38813559322033897</v>
+        <v>0.39152542372881355</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52146,11 +52185,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G701)</f>
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E5/COUNTA(Roster!A2:A701))</f>
-        <v>0.52711864406779663</v>
+        <v>0.53559322033898304</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52168,11 +52207,11 @@
       </c>
       <c r="E6" s="8">
         <f>COUNTA(Roster!H2:H701)</f>
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F6" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E6/COUNTA(Roster!A2:A701))</f>
-        <v>0.764406779661017</v>
+        <v>0.76779661016949152</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
@@ -52190,11 +52229,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I701)</f>
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E7/COUNTA(Roster!A2:A701))</f>
-        <v>0.53050847457627115</v>
+        <v>0.53559322033898304</v>
       </c>
     </row>
   </sheetData>
@@ -52237,11 +52276,11 @@
       </c>
       <c r="C2" s="6">
         <f>COUNTIF(Roster!$I$2:$I$701,A2)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.6677316293929709E-2</v>
+        <v>7.9113924050632917E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52253,11 +52292,11 @@
       </c>
       <c r="C3" s="6">
         <f>COUNTIF(Roster!$I$2:$I$701,A3)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.12140575079872204</v>
+        <v>0.12341772151898735</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52273,7 +52312,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.5846645367412137E-2</v>
+        <v>9.49367088607595E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52289,7 +52328,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>7.0287539936102233E-2</v>
+        <v>6.9620253164556958E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52305,7 +52344,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.12140575079872204</v>
+        <v>0.12025316455696203</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52321,7 +52360,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13418530351437699</v>
+        <v>0.13291139240506328</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -52337,7 +52376,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10223642172523961</v>
+        <v>0.10126582278481013</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -52349,11 +52388,11 @@
       </c>
       <c r="C9" s="6">
         <f>COUNTIF(Roster!$I$2:$I$701,A9)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10543130990415335</v>
+        <v>0.10759493670886076</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -52369,7 +52408,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.7092651757188496E-2</v>
+        <v>6.6455696202531639E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -52385,7 +52424,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.8338658146964855E-2</v>
+        <v>3.7974683544303799E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -52401,7 +52440,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.8338658146964855E-2</v>
+        <v>3.7974683544303799E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -52417,7 +52456,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.8753993610223641E-2</v>
+        <v>2.8481012658227847E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -52426,7 +52465,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -52565,7 +52604,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q701,"Yes")</f>
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1740</v>
@@ -52577,7 +52616,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>0.7</v>
+        <v>0.7533333333333333</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1740</v>
@@ -52589,7 +52628,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P701),0)</f>
-        <v>3.1322033898305084</v>
+        <v>3.1610169491525424</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1740</v>

</xml_diff>

<commit_message>
Fixed some F capes
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851A60DF-75E6-4CAD-972E-9026055D9E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDF6A86-3E05-48FC-91EC-80CCD93E6DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9406" uniqueCount="1874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9423" uniqueCount="1875">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5674,6 +5674,9 @@
   </si>
   <si>
     <t>Non-cape</t>
+  </si>
+  <si>
+    <t>Shaker, Master</t>
   </si>
 </sst>
 </file>
@@ -14914,7 +14917,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="8" max="8" width="29.42578125" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
     <col min="11" max="11" width="28" customWidth="1"/>
@@ -23514,9 +23517,15 @@
       <c r="C147" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D147" s="5"/>
-      <c r="E147" s="5"/>
-      <c r="F147" s="5"/>
+      <c r="D147" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E147" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F147" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G147" s="5" t="s">
         <v>47</v>
       </c>
@@ -23538,11 +23547,11 @@
       <c r="O147" s="5"/>
       <c r="P147" s="6">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q147" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R147" s="5" t="s">
         <v>51</v>
@@ -23576,13 +23585,17 @@
       <c r="D148" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E148" s="5"/>
+      <c r="E148" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F148" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G148" s="5"/>
+      <c r="G148" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H148" s="5" t="s">
-        <v>149</v>
+        <v>77</v>
       </c>
       <c r="I148" s="5" t="s">
         <v>71</v>
@@ -23601,11 +23614,11 @@
       <c r="O148" s="5"/>
       <c r="P148" s="6">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q148" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R148" s="5" t="s">
         <v>51</v>
@@ -24769,8 +24782,12 @@
       <c r="H169" s="5" t="s">
         <v>1871</v>
       </c>
-      <c r="I169" s="5"/>
-      <c r="J169" s="5"/>
+      <c r="I169" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J169" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="K169" s="5"/>
       <c r="L169" s="5"/>
       <c r="M169" s="5"/>
@@ -24780,11 +24797,11 @@
       <c r="O169" s="5"/>
       <c r="P169" s="6">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q169" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R169" s="5" t="s">
         <v>51</v>
@@ -25018,7 +25035,9 @@
       <c r="F174" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G174" s="5"/>
+      <c r="G174" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="H174" s="5" t="s">
         <v>664</v>
       </c>
@@ -25037,11 +25056,11 @@
       <c r="O174" s="5"/>
       <c r="P174" s="6">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q174" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R174" s="5" t="s">
         <v>51</v>
@@ -25519,7 +25538,9 @@
       <c r="F183" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G183" s="5"/>
+      <c r="G183" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="H183" s="5" t="s">
         <v>323</v>
       </c>
@@ -25538,11 +25559,11 @@
       <c r="O183" s="5"/>
       <c r="P183" s="6">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q183" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R183" s="5" t="s">
         <v>51</v>
@@ -26123,8 +26144,12 @@
       <c r="H193" s="5" t="s">
         <v>720</v>
       </c>
-      <c r="I193" s="5"/>
-      <c r="J193" s="5"/>
+      <c r="I193" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J193" s="5" t="s">
+        <v>1874</v>
+      </c>
       <c r="K193" s="5"/>
       <c r="L193" s="5"/>
       <c r="M193" s="5"/>
@@ -26134,11 +26159,11 @@
       <c r="O193" s="5"/>
       <c r="P193" s="6">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q193" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R193" s="5" t="s">
         <v>51</v>
@@ -26334,7 +26359,9 @@
       <c r="I197" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="J197" s="5"/>
+      <c r="J197" s="5" t="s">
+        <v>192</v>
+      </c>
       <c r="K197" s="5" t="s">
         <v>119</v>
       </c>
@@ -26388,16 +26415,24 @@
       <c r="D198" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="5"/>
+      <c r="E198" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F198" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G198" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H198" s="5" t="s">
         <v>58</v>
       </c>
       <c r="I198" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="J198" s="5"/>
+      <c r="J198" s="5" t="s">
+        <v>78</v>
+      </c>
       <c r="K198" s="5" t="s">
         <v>133</v>
       </c>
@@ -26409,11 +26444,11 @@
       <c r="O198" s="5"/>
       <c r="P198" s="6">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q198" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R198" s="5" t="s">
         <v>51</v>
@@ -26544,7 +26579,9 @@
       <c r="C201" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D201" s="5"/>
+      <c r="D201" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="E201" s="5" t="s">
         <v>45</v>
       </c>
@@ -26576,11 +26613,11 @@
       </c>
       <c r="P201" s="6">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q201" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R201" s="5" t="s">
         <v>51</v>
@@ -52119,11 +52156,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D701)</f>
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E2/COUNTA(Roster!A2:A701))</f>
-        <v>0.54067796610169494</v>
+        <v>0.54406779661016946</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -52141,11 +52178,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E701)</f>
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E3/COUNTA(Roster!A2:A701))</f>
-        <v>0.38983050847457629</v>
+        <v>0.39491525423728813</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52163,11 +52200,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F701)</f>
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E4/COUNTA(Roster!A2:A701))</f>
-        <v>0.39152542372881355</v>
+        <v>0.39491525423728813</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52185,11 +52222,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G701)</f>
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E5/COUNTA(Roster!A2:A701))</f>
-        <v>0.53559322033898304</v>
+        <v>0.5423728813559322</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52229,11 +52266,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I701)</f>
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E7/COUNTA(Roster!A2:A701))</f>
-        <v>0.53559322033898304</v>
+        <v>0.53898305084745768</v>
       </c>
     </row>
   </sheetData>
@@ -52280,7 +52317,7 @@
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.9113924050632917E-2</v>
+        <v>7.8616352201257858E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52296,7 +52333,7 @@
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.12341772151898735</v>
+        <v>0.12264150943396226</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52312,7 +52349,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.49367088607595E-2</v>
+        <v>9.4339622641509441E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52328,7 +52365,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>6.9620253164556958E-2</v>
+        <v>6.9182389937106917E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52344,7 +52381,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.12025316455696203</v>
+        <v>0.11949685534591195</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52360,7 +52397,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13291139240506328</v>
+        <v>0.13207547169811321</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -52372,11 +52409,11 @@
       </c>
       <c r="C8" s="6">
         <f>COUNTIF(Roster!$I$2:$I$701,A8)</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10126582278481013</v>
+        <v>0.1069182389937107</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -52392,7 +52429,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10759493670886076</v>
+        <v>0.1069182389937107</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -52408,7 +52445,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.6455696202531639E-2</v>
+        <v>6.6037735849056603E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -52424,7 +52461,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.7974683544303799E-2</v>
+        <v>3.7735849056603772E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -52440,7 +52477,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.7974683544303799E-2</v>
+        <v>3.7735849056603772E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -52456,7 +52493,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.8481012658227847E-2</v>
+        <v>2.8301886792452831E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -52465,7 +52502,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -52604,7 +52641,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q701,"Yes")</f>
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1740</v>
@@ -52616,7 +52653,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>0.7533333333333333</v>
+        <v>0.80666666666666664</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1740</v>
@@ -52628,7 +52665,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P701),0)</f>
-        <v>3.1610169491525424</v>
+        <v>3.1830508474576269</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1740</v>

</xml_diff>

<commit_message>
Corrected more post Ward capes
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF6E682-F2AF-41D5-B09B-10C8CCD077E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8EA23C-DFE8-4D8F-A0FB-3A08FFF18A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="2805" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9457" uniqueCount="1876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9465" uniqueCount="1879">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5680,6 +5680,15 @@
   </si>
   <si>
     <t>Unicorn IV</t>
+  </si>
+  <si>
+    <t>The Flock</t>
+  </si>
+  <si>
+    <t>Erring Right</t>
+  </si>
+  <si>
+    <t>The Shepherds</t>
   </si>
 </sst>
 </file>
@@ -19950,7 +19959,7 @@
         <v>57</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>58</v>
+        <v>1876</v>
       </c>
       <c r="I86" s="5" t="s">
         <v>192</v>
@@ -20335,9 +20344,15 @@
       <c r="D93" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-      <c r="G93" s="5"/>
+      <c r="E93" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>1865</v>
+      </c>
       <c r="H93" s="5" t="s">
         <v>77</v>
       </c>
@@ -20352,7 +20367,7 @@
       <c r="O93" s="5"/>
       <c r="P93" s="6">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q93" s="6" t="str">
         <f t="shared" si="3"/>
@@ -21298,10 +21313,10 @@
         <v>46</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="H109" s="5" t="s">
-        <v>83</v>
+        <v>1876</v>
       </c>
       <c r="I109" s="5" t="s">
         <v>78</v>
@@ -26210,7 +26225,7 @@
         <v>57</v>
       </c>
       <c r="H194" s="5" t="s">
-        <v>319</v>
+        <v>1876</v>
       </c>
       <c r="I194" s="5"/>
       <c r="J194" s="5"/>
@@ -28013,10 +28028,10 @@
         <v>46</v>
       </c>
       <c r="G226" s="5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="H226" s="5" t="s">
-        <v>272</v>
+        <v>1876</v>
       </c>
       <c r="I226" s="5" t="s">
         <v>91</v>
@@ -31037,10 +31052,10 @@
         <v>46</v>
       </c>
       <c r="G280" s="5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="H280" s="5" t="s">
-        <v>83</v>
+        <v>1876</v>
       </c>
       <c r="I280" s="5" t="s">
         <v>123</v>
@@ -32171,7 +32186,7 @@
         <v>57</v>
       </c>
       <c r="H301" s="5" t="s">
-        <v>323</v>
+        <v>1877</v>
       </c>
       <c r="I301" s="5" t="s">
         <v>119</v>
@@ -40654,13 +40669,21 @@
       <c r="C453" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D453" s="5"/>
-      <c r="E453" s="5"/>
-      <c r="F453" s="5"/>
+      <c r="D453" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E453" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F453" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G453" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="H453" s="5"/>
+        <v>57</v>
+      </c>
+      <c r="H453" s="5" t="s">
+        <v>1876</v>
+      </c>
       <c r="I453" s="5" t="s">
         <v>49</v>
       </c>
@@ -40676,11 +40699,11 @@
       <c r="O453" s="5"/>
       <c r="P453" s="6">
         <f t="shared" si="14"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q453" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R453" s="5" t="s">
         <v>125</v>
@@ -40769,7 +40792,9 @@
       <c r="D455" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E455" s="5"/>
+      <c r="E455" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F455" s="5" t="s">
         <v>107</v>
       </c>
@@ -40777,7 +40802,7 @@
         <v>57</v>
       </c>
       <c r="H455" s="5" t="s">
-        <v>96</v>
+        <v>1878</v>
       </c>
       <c r="I455" s="5" t="s">
         <v>78</v>
@@ -40794,11 +40819,11 @@
       <c r="O455" s="5"/>
       <c r="P455" s="6">
         <f t="shared" si="14"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q455" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R455" s="5" t="s">
         <v>51</v>
@@ -52227,11 +52252,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D701)</f>
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E2/COUNTA(Roster!A2:A701))</f>
-        <v>0.54915254237288136</v>
+        <v>0.55084745762711862</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -52249,11 +52274,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E701)</f>
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E3/COUNTA(Roster!A2:A701))</f>
-        <v>0.4152542372881356</v>
+        <v>0.42033898305084744</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52271,11 +52296,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F701)</f>
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E4/COUNTA(Roster!A2:A701))</f>
-        <v>0.41186440677966102</v>
+        <v>0.4152542372881356</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52293,11 +52318,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G701)</f>
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E5/COUNTA(Roster!A2:A701))</f>
-        <v>0.54915254237288136</v>
+        <v>0.55084745762711862</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52315,11 +52340,11 @@
       </c>
       <c r="E6" s="8">
         <f>COUNTA(Roster!H2:H701)</f>
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F6" s="9">
         <f>IF(COUNTA(Roster!A2:A701)=0,0,E6/COUNTA(Roster!A2:A701))</f>
-        <v>0.76949152542372878</v>
+        <v>0.77118644067796616</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
@@ -52712,7 +52737,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q701,"Yes")</f>
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1740</v>
@@ -52724,7 +52749,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>0.91333333333333333</v>
+        <v>0.92666666666666664</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1740</v>
@@ -52736,7 +52761,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P701),0)</f>
-        <v>3.2355932203389832</v>
+        <v>3.2491525423728813</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1740</v>

</xml_diff>

<commit_message>
Redraw the whole schedule and reset at each player's local midnight
- New --redraw build option re-draws every day, past ones included, as a new
  schedule edition (now edition 2); the site clears results from the old
  edition and shows a one-time note explaining why
- Reset time is now "Midnight local time": puzzle numbers follow the
  player's own calendar date, and the page rolls over at local midnight
  (also checked when the tab becomes visible again)
- Frozen window widened to two days past UTC so players up to UTC+14 never
  see an answer change
- Workbook Settings/Rules text and README updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2rJagsxGbYcrTNoNQYqhz
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -5259,10 +5259,10 @@
     <t>Reset time</t>
   </si>
   <si>
-    <t>Midnight CET</t>
-  </si>
-  <si>
-    <t>As on Eldendle</t>
+    <t>Midnight local time</t>
+  </si>
+  <si>
+    <t>Each player's own midnight, as on Wordle</t>
   </si>
   <si>
     <t>— Live progress —</t>
@@ -5316,7 +5316,7 @@
     <t>Daily seed</t>
   </si>
   <si>
-    <t>Deterministic daily puzzle; resets midnight CET; progress in local storage.</t>
+    <t>Deterministic daily puzzle; resets at each player's local midnight; progress in local storage.</t>
   </si>
   <si>
     <t>Alias handling</t>

</xml_diff>

<commit_message>
Updated Snag and Screamer
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66D0E0F-5769-40F5-9405-AA9D170AB080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABEB360-545A-4B00-858A-2B9A0447D273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9563" uniqueCount="1904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9573" uniqueCount="1907">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5764,6 +5764,15 @@
   </si>
   <si>
     <t>The Wardens</t>
+  </si>
+  <si>
+    <t>The Mall Cluster</t>
+  </si>
+  <si>
+    <t>Blaster, Striker</t>
+  </si>
+  <si>
+    <t>Grab-bag cape. Can treat any direction as down which allowed him to leap without jumping movement. Can create large gauntlets that fit over his arms. Can force negative emotions on people he touches with his gauntlets or apply dedicated emotions from his tinkered projectiles. Can punch through inorganic materials.</t>
   </si>
 </sst>
 </file>
@@ -41527,8 +41536,12 @@
       <c r="D465" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E465" s="5"/>
-      <c r="F465" s="5"/>
+      <c r="E465" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F465" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G465" s="5" t="s">
         <v>47</v>
       </c>
@@ -41550,11 +41563,11 @@
       <c r="O465" s="5"/>
       <c r="P465" s="6">
         <f t="shared" si="14"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q465" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R465" s="5" t="s">
         <v>51</v>
@@ -42908,15 +42921,27 @@
       <c r="C489" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D489" s="5"/>
-      <c r="E489" s="5"/>
-      <c r="F489" s="5"/>
+      <c r="D489" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E489" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F489" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G489" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H489" s="5"/>
-      <c r="I489" s="5"/>
-      <c r="J489" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="H489" s="5" t="s">
+        <v>1904</v>
+      </c>
+      <c r="I489" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="J489" s="5" t="s">
+        <v>1905</v>
+      </c>
       <c r="K489" s="5"/>
       <c r="L489" s="5"/>
       <c r="M489" s="5"/>
@@ -42926,20 +42951,24 @@
       <c r="O489" s="5"/>
       <c r="P489" s="6">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q489" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R489" s="5" t="s">
         <v>51</v>
       </c>
       <c r="S489" s="5"/>
-      <c r="T489" s="5"/>
-      <c r="U489" s="5"/>
+      <c r="T489" s="5" t="s">
+        <v>1906</v>
+      </c>
+      <c r="U489" s="5" t="s">
+        <v>1904</v>
+      </c>
       <c r="V489" s="5" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="W489" s="5" t="s">
         <v>128</v>
@@ -52659,11 +52688,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D705)</f>
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E2/COUNTA(Roster!A2:A705))</f>
-        <v>0.55892255892255893</v>
+        <v>0.56060606060606055</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -52681,11 +52710,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E705)</f>
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E3/COUNTA(Roster!A2:A705))</f>
-        <v>0.43265993265993263</v>
+        <v>0.43602693602693604</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52703,11 +52732,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F705)</f>
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E4/COUNTA(Roster!A2:A705))</f>
-        <v>0.42760942760942761</v>
+        <v>0.43097643097643096</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52747,11 +52776,11 @@
       </c>
       <c r="E6" s="8">
         <f>COUNTA(Roster!H2:H705)</f>
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F6" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E6/COUNTA(Roster!A2:A705))</f>
-        <v>0.77441077441077444</v>
+        <v>0.77609427609427606</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
@@ -52769,11 +52798,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I705)</f>
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E7/COUNTA(Roster!A2:A705))</f>
-        <v>0.54882154882154888</v>
+        <v>0.5505050505050505</v>
       </c>
     </row>
   </sheetData>
@@ -52820,7 +52849,7 @@
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.9754601226993863E-2</v>
+        <v>7.9510703363914373E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52836,7 +52865,7 @@
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.12576687116564417</v>
+        <v>0.12538226299694188</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52852,7 +52881,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.202453987730061E-2</v>
+        <v>9.1743119266055051E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52868,7 +52897,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>6.7484662576687116E-2</v>
+        <v>6.7278287461773695E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52884,7 +52913,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.1165644171779141</v>
+        <v>0.11620795107033639</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52896,11 +52925,11 @@
       </c>
       <c r="C7" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A7)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13496932515337423</v>
+        <v>0.13761467889908258</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -52916,7 +52945,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10736196319018405</v>
+        <v>0.10703363914373089</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -52932,7 +52961,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10429447852760736</v>
+        <v>0.10397553516819572</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -52948,7 +52977,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>7.0552147239263799E-2</v>
+        <v>7.0336391437308868E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -52964,7 +52993,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.6809815950920248E-2</v>
+        <v>3.669724770642202E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -52980,7 +53009,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.6809815950920248E-2</v>
+        <v>3.669724770642202E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -52996,7 +53025,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.7607361963190184E-2</v>
+        <v>2.7522935779816515E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -53005,7 +53034,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -53144,7 +53173,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q705,"Yes")</f>
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1739</v>
@@ -53156,7 +53185,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.0133333333333334</v>
+        <v>1.0266666666666666</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1739</v>
@@ -53168,7 +53197,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P705),0)</f>
-        <v>3.3047138047138045</v>
+        <v>3.3164983164983166</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1739</v>

</xml_diff>

<commit_message>
Updated Echidna, Coil and a few others
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABEB360-545A-4B00-858A-2B9A0447D273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C419EC-746C-4259-8B59-624CBFB11E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9573" uniqueCount="1907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9578" uniqueCount="1908">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5773,6 +5773,9 @@
   </si>
   <si>
     <t>Grab-bag cape. Can treat any direction as down which allowed him to leap without jumping movement. Can create large gauntlets that fit over his arms. Can force negative emotions on people he touches with his gauntlets or apply dedicated emotions from his tinkered projectiles. Can punch through inorganic materials.</t>
+  </si>
+  <si>
+    <t>Stranger, Shaker</t>
   </si>
 </sst>
 </file>
@@ -21658,7 +21661,7 @@
         <v>47</v>
       </c>
       <c r="H113" s="5" t="s">
-        <v>58</v>
+        <v>224</v>
       </c>
       <c r="I113" s="5" t="s">
         <v>49</v>
@@ -21886,16 +21889,24 @@
       <c r="D117" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E117" s="5"/>
-      <c r="F117" s="5"/>
+      <c r="E117" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F117" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G117" s="5" t="s">
-        <v>57</v>
+        <v>1864</v>
       </c>
       <c r="H117" s="5" t="s">
         <v>494</v>
       </c>
-      <c r="I117" s="5"/>
-      <c r="J117" s="5"/>
+      <c r="I117" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J117" s="5" t="s">
+        <v>1907</v>
+      </c>
       <c r="K117" s="5"/>
       <c r="L117" s="5"/>
       <c r="M117" s="5"/>
@@ -21905,11 +21916,11 @@
       <c r="O117" s="5"/>
       <c r="P117" s="6">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q117" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R117" s="5" t="s">
         <v>51</v>
@@ -22189,9 +22200,11 @@
       <c r="F122" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G122" s="5"/>
+      <c r="G122" s="5" t="s">
+        <v>1864</v>
+      </c>
       <c r="H122" s="5" t="s">
-        <v>96</v>
+        <v>1136</v>
       </c>
       <c r="I122" s="5" t="s">
         <v>59</v>
@@ -22208,11 +22221,11 @@
       <c r="O122" s="5"/>
       <c r="P122" s="6">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q122" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R122" s="5" t="s">
         <v>51</v>
@@ -23849,7 +23862,7 @@
         <v>47</v>
       </c>
       <c r="H150" s="5" t="s">
-        <v>77</v>
+        <v>214</v>
       </c>
       <c r="I150" s="5" t="s">
         <v>78</v>
@@ -52710,11 +52723,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E705)</f>
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E3/COUNTA(Roster!A2:A705))</f>
-        <v>0.43602693602693604</v>
+        <v>0.43771043771043772</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52732,11 +52745,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F705)</f>
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E4/COUNTA(Roster!A2:A705))</f>
-        <v>0.43097643097643096</v>
+        <v>0.43265993265993263</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52754,11 +52767,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G705)</f>
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E5/COUNTA(Roster!A2:A705))</f>
-        <v>0.56228956228956228</v>
+        <v>0.56397306397306401</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52798,11 +52811,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I705)</f>
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E7/COUNTA(Roster!A2:A705))</f>
-        <v>0.5505050505050505</v>
+        <v>0.55218855218855223</v>
       </c>
     </row>
   </sheetData>
@@ -52845,11 +52858,11 @@
       </c>
       <c r="C2" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A2)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.9510703363914373E-2</v>
+        <v>8.2317073170731711E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52865,7 +52878,7 @@
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.12538226299694188</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52881,7 +52894,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.1743119266055051E-2</v>
+        <v>9.1463414634146339E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52897,7 +52910,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>6.7278287461773695E-2</v>
+        <v>6.7073170731707321E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52913,7 +52926,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.11620795107033639</v>
+        <v>0.11585365853658537</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52929,7 +52942,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13761467889908258</v>
+        <v>0.13719512195121952</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -52945,7 +52958,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10703363914373089</v>
+        <v>0.10670731707317073</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -52961,7 +52974,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10397553516819572</v>
+        <v>0.10365853658536585</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -52977,7 +52990,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>7.0336391437308868E-2</v>
+        <v>7.0121951219512202E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -52993,7 +53006,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.669724770642202E-2</v>
+        <v>3.6585365853658534E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -53009,7 +53022,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.669724770642202E-2</v>
+        <v>3.6585365853658534E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -53025,7 +53038,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.7522935779816515E-2</v>
+        <v>2.7439024390243903E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -53034,7 +53047,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -53173,7 +53186,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q705,"Yes")</f>
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1739</v>
@@ -53185,7 +53198,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.0266666666666666</v>
+        <v>1.04</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1739</v>
@@ -53197,7 +53210,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P705),0)</f>
-        <v>3.3164983164983166</v>
+        <v>3.3232323232323231</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1739</v>

</xml_diff>

<commit_message>
Updated Wanton and Winter
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2152F47-E54C-4CFF-97C1-0F9010868C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22B0D38-A59F-48BD-BA99-1FCDE949E3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5925" yWindow="4785" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9578" uniqueCount="1907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9586" uniqueCount="1909">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5773,6 +5773,12 @@
   </si>
   <si>
     <t>Stranger, Shaker</t>
+  </si>
+  <si>
+    <t>Unknown powers. Tended to hold his abilities back to avoid scaring people.</t>
+  </si>
+  <si>
+    <t>Andrew Hawke</t>
   </si>
 </sst>
 </file>
@@ -47801,7 +47807,9 @@
       <c r="G575" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H575" s="5"/>
+      <c r="H575" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="I575" s="5"/>
       <c r="J575" s="5"/>
       <c r="K575" s="5"/>
@@ -47813,7 +47821,7 @@
       <c r="O575" s="5"/>
       <c r="P575" s="6">
         <f t="shared" si="18"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q575" s="6" t="str">
         <f t="shared" si="17"/>
@@ -47822,8 +47830,12 @@
       <c r="R575" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="S575" s="5"/>
-      <c r="T575" s="5"/>
+      <c r="S575" s="5" t="s">
+        <v>1908</v>
+      </c>
+      <c r="T575" s="5" t="s">
+        <v>1907</v>
+      </c>
       <c r="U575" s="5"/>
       <c r="V575" s="5" t="s">
         <v>47</v>
@@ -48124,9 +48136,15 @@
       <c r="D581" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E581" s="5"/>
-      <c r="F581" s="5"/>
-      <c r="G581" s="5"/>
+      <c r="E581" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F581" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G581" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="H581" s="5" t="s">
         <v>83</v>
       </c>
@@ -48147,11 +48165,11 @@
       <c r="O581" s="5"/>
       <c r="P581" s="6">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q581" s="6" t="str">
         <f t="shared" si="19"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R581" s="5" t="s">
         <v>51</v>
@@ -48450,7 +48468,9 @@
       <c r="D587" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E587" s="5"/>
+      <c r="E587" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F587" s="5" t="s">
         <v>107</v>
       </c>
@@ -48461,11 +48481,11 @@
         <v>1131</v>
       </c>
       <c r="I587" s="5" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="J587" s="5"/>
       <c r="K587" s="5" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="L587" s="5"/>
       <c r="M587" s="5"/>
@@ -48475,11 +48495,11 @@
       <c r="O587" s="5"/>
       <c r="P587" s="6">
         <f t="shared" si="18"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q587" s="6" t="str">
         <f t="shared" si="19"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R587" s="5" t="s">
         <v>51</v>
@@ -48674,7 +48694,9 @@
       <c r="D591" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E591" s="5"/>
+      <c r="E591" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F591" s="5" t="s">
         <v>107</v>
       </c>
@@ -48699,11 +48721,11 @@
       <c r="O591" s="5"/>
       <c r="P591" s="6">
         <f t="shared" si="18"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q591" s="6" t="str">
         <f t="shared" si="19"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R591" s="5" t="s">
         <v>51</v>
@@ -52720,11 +52742,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E705)</f>
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E3/COUNTA(Roster!A2:A705))</f>
-        <v>0.43771043771043772</v>
+        <v>0.44276094276094274</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52742,11 +52764,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F705)</f>
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E4/COUNTA(Roster!A2:A705))</f>
-        <v>0.43265993265993263</v>
+        <v>0.43434343434343436</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52764,11 +52786,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G705)</f>
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E5/COUNTA(Roster!A2:A705))</f>
-        <v>0.56397306397306401</v>
+        <v>0.56565656565656564</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52786,11 +52808,11 @@
       </c>
       <c r="E6" s="8">
         <f>COUNTA(Roster!H2:H705)</f>
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F6" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E6/COUNTA(Roster!A2:A705))</f>
-        <v>0.77609427609427606</v>
+        <v>0.77777777777777779</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
@@ -52871,11 +52893,11 @@
       </c>
       <c r="C3" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A3)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.12804878048780488</v>
+        <v>0.13109756097560976</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52983,11 +53005,11 @@
       </c>
       <c r="C10" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A10)</f>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>7.0121951219512202E-2</v>
+        <v>6.7073170731707321E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -53183,7 +53205,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q705,"Yes")</f>
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1738</v>
@@ -53195,7 +53217,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1738</v>
@@ -53207,7 +53229,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P705),0)</f>
-        <v>3.3232323232323231</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1738</v>

</xml_diff>

<commit_message>
Updated Moonsong, Mouse Protector, Newter
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22B0D38-A59F-48BD-BA99-1FCDE949E3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA572BE7-7B18-4A06-93ED-DEC5A07921F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9060" yWindow="4110" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9586" uniqueCount="1909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9599" uniqueCount="1911">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5779,6 +5779,12 @@
   </si>
   <si>
     <t>Andrew Hawke</t>
+  </si>
+  <si>
+    <t>A gravity manipulator who can create multiple conflicting gravity fields within an area, alongside a thinker-aspect that allows her to perceive gravity wells.</t>
+  </si>
+  <si>
+    <t>Brianna</t>
   </si>
 </sst>
 </file>
@@ -26810,7 +26816,7 @@
         <v>214</v>
       </c>
       <c r="I202" s="5" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="J202" s="5"/>
       <c r="K202" s="5" t="s">
@@ -29967,10 +29973,10 @@
         <v>313</v>
       </c>
       <c r="I257" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="J257" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="J257" s="5" t="s">
-        <v>78</v>
       </c>
       <c r="K257" s="5" t="s">
         <v>894</v>
@@ -34901,17 +34907,27 @@
       <c r="C345" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D345" s="5"/>
-      <c r="E345" s="5"/>
-      <c r="F345" s="5"/>
+      <c r="D345" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E345" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G345" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H345" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="I345" s="5"/>
-      <c r="J345" s="5"/>
+        <v>1876</v>
+      </c>
+      <c r="I345" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J345" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="K345" s="5"/>
       <c r="L345" s="5"/>
       <c r="M345" s="5"/>
@@ -34921,17 +34937,21 @@
       <c r="O345" s="5"/>
       <c r="P345" s="6">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q345" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R345" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="S345" s="5"/>
-      <c r="T345" s="5"/>
+      <c r="S345" s="5" t="s">
+        <v>1910</v>
+      </c>
+      <c r="T345" s="5" t="s">
+        <v>1909</v>
+      </c>
       <c r="U345" s="5" t="s">
         <v>318</v>
       </c>
@@ -34957,8 +34977,12 @@
       <c r="D346" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E346" s="5"/>
-      <c r="F346" s="5"/>
+      <c r="E346" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F346" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G346" s="5" t="s">
         <v>57</v>
       </c>
@@ -34980,11 +35004,11 @@
       <c r="O346" s="5"/>
       <c r="P346" s="6">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q346" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R346" s="5" t="s">
         <v>51</v>
@@ -35116,8 +35140,12 @@
       <c r="D349" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E349" s="5"/>
-      <c r="F349" s="5"/>
+      <c r="E349" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F349" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G349" s="5" t="s">
         <v>47</v>
       </c>
@@ -35127,7 +35155,9 @@
       <c r="I349" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="J349" s="5"/>
+      <c r="J349" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="K349" s="5" t="s">
         <v>71</v>
       </c>
@@ -35139,11 +35169,11 @@
       <c r="O349" s="5"/>
       <c r="P349" s="6">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q349" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R349" s="5" t="s">
         <v>51</v>
@@ -35785,7 +35815,9 @@
       <c r="E361" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="F361" s="5"/>
+      <c r="F361" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G361" s="5" t="s">
         <v>57</v>
       </c>
@@ -35809,11 +35841,11 @@
       <c r="O361" s="5"/>
       <c r="P361" s="6">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q361" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R361" s="5" t="s">
         <v>51</v>
@@ -52648,7 +52680,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>I2:I705</xm:sqref>
+          <xm:sqref>I2:I256 I258:I705 J257</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
@@ -52720,11 +52752,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D705)</f>
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E2/COUNTA(Roster!A2:A705))</f>
-        <v>0.56060606060606055</v>
+        <v>0.56228956228956228</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -52742,11 +52774,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E705)</f>
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E3/COUNTA(Roster!A2:A705))</f>
-        <v>0.44276094276094274</v>
+        <v>0.44781144781144783</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52764,11 +52796,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F705)</f>
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E4/COUNTA(Roster!A2:A705))</f>
-        <v>0.43434343434343436</v>
+        <v>0.44107744107744107</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52830,11 +52862,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I705)</f>
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E7/COUNTA(Roster!A2:A705))</f>
-        <v>0.55218855218855223</v>
+        <v>0.55387205387205385</v>
       </c>
     </row>
   </sheetData>
@@ -52881,7 +52913,7 @@
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.926829268292683E-2</v>
+        <v>7.9027355623100301E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52893,11 +52925,11 @@
       </c>
       <c r="C3" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A3)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.13109756097560976</v>
+        <v>0.1337386018237082</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52913,7 +52945,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.1463414634146339E-2</v>
+        <v>9.1185410334346503E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52929,7 +52961,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>6.7073170731707321E-2</v>
+        <v>6.6869300911854099E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52941,11 +52973,11 @@
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A6)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.11585365853658537</v>
+        <v>0.11854103343465046</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52961,7 +52993,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13719512195121952</v>
+        <v>0.13677811550151975</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -52977,7 +53009,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10670731707317073</v>
+        <v>0.10638297872340426</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -52989,11 +53021,11 @@
       </c>
       <c r="C9" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A9)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10365853658536585</v>
+        <v>0.10030395136778116</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -53005,11 +53037,11 @@
       </c>
       <c r="C10" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A10)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.7073170731707321E-2</v>
+        <v>6.9908814589665649E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -53021,11 +53053,11 @@
       </c>
       <c r="C11" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A11)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.6585365853658534E-2</v>
+        <v>3.3434650455927049E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -53041,7 +53073,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.6585365853658534E-2</v>
+        <v>3.64741641337386E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -53057,7 +53089,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.7439024390243903E-2</v>
+        <v>2.7355623100303952E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -53066,7 +53098,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -53205,7 +53237,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q705,"Yes")</f>
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1738</v>
@@ -53217,7 +53249,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.06</v>
+        <v>1.0866666666666667</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1738</v>
@@ -53229,7 +53261,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P705),0)</f>
-        <v>3.3333333333333335</v>
+        <v>3.3484848484848486</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1738</v>

</xml_diff>

<commit_message>
Updated Skitter and some unknowns statuses
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA572BE7-7B18-4A06-93ED-DEC5A07921F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8C4EE6-6A9F-4169-A65B-8B97BBEE42E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9060" yWindow="4110" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9599" uniqueCount="1911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9605" uniqueCount="1911">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -42450,19 +42450,29 @@
       </c>
       <c r="B480" s="5"/>
       <c r="C480" s="5" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="D480" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E480" s="5"/>
-      <c r="F480" s="5"/>
-      <c r="G480" s="5"/>
+      <c r="E480" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F480" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G480" s="5" t="s">
+        <v>1863</v>
+      </c>
       <c r="H480" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="I480" s="5"/>
-      <c r="J480" s="5"/>
+      <c r="I480" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J480" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="K480" s="5"/>
       <c r="L480" s="5"/>
       <c r="M480" s="5"/>
@@ -42472,11 +42482,11 @@
       <c r="O480" s="5"/>
       <c r="P480" s="6">
         <f t="shared" si="16"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q480" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R480" s="5" t="s">
         <v>51</v>
@@ -42728,7 +42738,9 @@
       <c r="F485" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G485" s="5"/>
+      <c r="G485" s="5" t="s">
+        <v>1863</v>
+      </c>
       <c r="H485" s="5" t="s">
         <v>313</v>
       </c>
@@ -42747,11 +42759,11 @@
       <c r="O485" s="5"/>
       <c r="P485" s="6">
         <f t="shared" si="16"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q485" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="R485" s="5" t="s">
         <v>51</v>
@@ -42792,7 +42804,7 @@
         <v>107</v>
       </c>
       <c r="G486" s="5" t="s">
-        <v>57</v>
+        <v>1863</v>
       </c>
       <c r="H486" s="5" t="s">
         <v>271</v>
@@ -52774,11 +52786,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E705)</f>
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E3/COUNTA(Roster!A2:A705))</f>
-        <v>0.44781144781144783</v>
+        <v>0.4494949494949495</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -52796,11 +52808,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F705)</f>
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E4/COUNTA(Roster!A2:A705))</f>
-        <v>0.44107744107744107</v>
+        <v>0.44276094276094274</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -52818,11 +52830,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G705)</f>
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E5/COUNTA(Roster!A2:A705))</f>
-        <v>0.56565656565656564</v>
+        <v>0.56902356902356899</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -52862,11 +52874,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I705)</f>
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A705)=0,0,E7/COUNTA(Roster!A2:A705))</f>
-        <v>0.55387205387205385</v>
+        <v>0.55555555555555558</v>
       </c>
     </row>
   </sheetData>
@@ -52913,7 +52925,7 @@
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.9027355623100301E-2</v>
+        <v>7.8787878787878782E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -52925,11 +52937,11 @@
       </c>
       <c r="C3" s="6">
         <f>COUNTIF(Roster!$I$2:$I$705,A3)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.1337386018237082</v>
+        <v>0.13636363636363635</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -52945,7 +52957,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.1185410334346503E-2</v>
+        <v>9.0909090909090912E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -52961,7 +52973,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>6.6869300911854099E-2</v>
+        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -52977,7 +52989,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.11854103343465046</v>
+        <v>0.11818181818181818</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -52993,7 +53005,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13677811550151975</v>
+        <v>0.13636363636363635</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -53009,7 +53021,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.10638297872340426</v>
+        <v>0.10606060606060606</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -53025,7 +53037,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10030395136778116</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -53041,7 +53053,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.9908814589665649E-2</v>
+        <v>6.9696969696969702E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -53057,7 +53069,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.3434650455927049E-2</v>
+        <v>3.3333333333333333E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -53073,7 +53085,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.64741641337386E-2</v>
+        <v>3.6363636363636362E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -53089,7 +53101,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>2.7355623100303952E-2</v>
+        <v>2.7272727272727271E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -53098,7 +53110,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -53237,7 +53249,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!Q2:Q705,"Yes")</f>
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1738</v>
@@ -53249,7 +53261,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.0866666666666667</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1738</v>
@@ -53261,7 +53273,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!P2:P705),0)</f>
-        <v>3.3484848484848486</v>
+        <v>3.3569023569023568</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1738</v>

</xml_diff>

<commit_message>
Updated Grue and Oni Lee
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189AE06D-8D7B-4B9E-BDAE-478F74A5D07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA42B26E-640E-4020-8161-9A07B4F9C2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9060" yWindow="4110" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9606" uniqueCount="1909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9607" uniqueCount="1909">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -27953,7 +27953,7 @@
         <v>43</v>
       </c>
       <c r="D222" s="5" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="E222" s="5" t="s">
         <v>45</v>
@@ -36843,7 +36843,9 @@
       <c r="I378" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="J378" s="5"/>
+      <c r="J378" s="5" t="s">
+        <v>192</v>
+      </c>
       <c r="K378" s="5" t="s">
         <v>71</v>
       </c>

</xml_diff>

<commit_message>
Updated some T capes
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03749663-F347-48FA-BD38-598517332492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2253BCF-D330-44A5-B603-A5723D9972E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5910" yWindow="5340" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10532" uniqueCount="1970">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10539" uniqueCount="1972">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5962,6 +5962,12 @@
   </si>
   <si>
     <t>Increased flexibility, strength, reflexes, durability, etc. Can teleport to anyone she's harmed and has the ability to prevent inflicted wounds from healing.</t>
+  </si>
+  <si>
+    <t>Power granter who could turn a person into a specialist by granting them extraordinary and inhuman levels of skill in an unconventional thing/tool/weapon, in exchange for their sanity and free will.</t>
+  </si>
+  <si>
+    <t>Case 70, can exist simultaneously and get past bars by touch teleportation.</t>
   </si>
 </sst>
 </file>
@@ -17736,7 +17742,9 @@
       <c r="F39" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G39" s="5"/>
+      <c r="G39" s="5" t="s">
+        <v>1845</v>
+      </c>
       <c r="H39" s="5" t="s">
         <v>90</v>
       </c>
@@ -17751,14 +17759,16 @@
       </c>
       <c r="L39" s="6">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M39" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="N39" s="5"/>
-      <c r="O39" s="5"/>
+      <c r="O39" s="5" t="s">
+        <v>1970</v>
+      </c>
       <c r="P39" s="5" t="s">
         <v>105</v>
       </c>
@@ -47542,30 +47552,40 @@
       <c r="C532" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D532" s="5"/>
-      <c r="E532" s="5"/>
-      <c r="F532" s="5"/>
+      <c r="D532" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E532" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F532" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="G532" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H532" s="5" t="s">
         <v>1406</v>
       </c>
-      <c r="I532" s="5"/>
+      <c r="I532" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="J532" s="5"/>
       <c r="K532" s="18" t="s">
         <v>1931</v>
       </c>
       <c r="L532" s="6">
         <f t="shared" ref="L532:L595" si="20">IF(A532="","",COUNTA(D532:F532)+COUNTA(G532:G532)+COUNTA(H532:H532)+COUNTA(I532:I532))</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M532" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="N532" s="5"/>
-      <c r="O532" s="5"/>
+      <c r="O532" s="5" t="s">
+        <v>1971</v>
+      </c>
       <c r="P532" s="5" t="s">
         <v>128</v>
       </c>
@@ -55773,11 +55793,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D715)</f>
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E2/COUNTA(Roster!A2:A715))</f>
-        <v>0.58940397350993379</v>
+        <v>0.59105960264900659</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -55795,11 +55815,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E715)</f>
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E3/COUNTA(Roster!A2:A715))</f>
-        <v>0.51986754966887416</v>
+        <v>0.52152317880794707</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -55817,11 +55837,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F715)</f>
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E4/COUNTA(Roster!A2:A715))</f>
-        <v>0.50331125827814571</v>
+        <v>0.50496688741721851</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -55839,11 +55859,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G715)</f>
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E5/COUNTA(Roster!A2:A715))</f>
-        <v>0.6258278145695364</v>
+        <v>0.62748344370860931</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -55883,11 +55903,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I715)</f>
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E7/COUNTA(Roster!A2:A715))</f>
-        <v>0.58443708609271527</v>
+        <v>0.58609271523178808</v>
       </c>
     </row>
   </sheetData>
@@ -55930,11 +55950,11 @@
       </c>
       <c r="C2" s="6">
         <f>COUNTIF(Roster!$I$2:$I$715,A2)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.6487252124645896E-2</v>
+        <v>7.909604519774012E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -55950,7 +55970,7 @@
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.1359773371104816</v>
+        <v>0.13559322033898305</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -55966,7 +55986,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.0651558073654395E-2</v>
+        <v>9.03954802259887E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -55982,7 +56002,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>5.6657223796033995E-2</v>
+        <v>5.6497175141242938E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -55998,7 +56018,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.11898016997167139</v>
+        <v>0.11864406779661017</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -56014,7 +56034,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.13031161473087818</v>
+        <v>0.12994350282485875</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -56030,7 +56050,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.11048158640226628</v>
+        <v>0.11016949152542373</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -56046,7 +56066,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10764872521246459</v>
+        <v>0.10734463276836158</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -56062,7 +56082,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.5155807365439092E-2</v>
+        <v>6.4971751412429377E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -56078,7 +56098,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.39943342776204E-2</v>
+        <v>3.3898305084745763E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -56094,7 +56114,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.9660056657223795E-2</v>
+        <v>3.954802259887006E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -56110,7 +56130,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>3.39943342776204E-2</v>
+        <v>3.3898305084745763E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -56119,7 +56139,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -56258,7 +56278,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!M2:M715,"Yes")</f>
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1720</v>
@@ -56270,7 +56290,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.5133333333333334</v>
+        <v>1.5266666666666666</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1720</v>
@@ -56282,7 +56302,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!L2:L715),0)</f>
-        <v>3.6175496688741724</v>
+        <v>3.6258278145695364</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1720</v>

</xml_diff>

<commit_message>
Updated Shuffle and Shortcut
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2253BCF-D330-44A5-B603-A5723D9972E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8386FCF8-958A-4767-9B7E-50149F7CB0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5910" yWindow="5340" windowWidth="28800" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10539" uniqueCount="1972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10547" uniqueCount="1973">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -5968,6 +5968,9 @@
   </si>
   <si>
     <t>Case 70, can exist simultaneously and get past bars by touch teleportation.</t>
+  </si>
+  <si>
+    <t>Controlled spatial distortion by drawing out circles with his polearm and then stepping on the affected space to propel himself forward.</t>
   </si>
 </sst>
 </file>
@@ -44698,30 +44701,40 @@
       <c r="C485" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D485" s="5"/>
-      <c r="E485" s="5"/>
-      <c r="F485" s="5"/>
+      <c r="D485" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E485" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F485" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G485" s="5" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="H485" s="5" t="s">
         <v>1406</v>
       </c>
-      <c r="I485" s="5"/>
+      <c r="I485" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="J485" s="5"/>
       <c r="K485" s="18" t="s">
         <v>1931</v>
       </c>
       <c r="L485" s="6">
         <f t="shared" si="16"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M485" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="N485" s="5"/>
-      <c r="O485" s="5"/>
+      <c r="O485" s="5" t="s">
+        <v>1972</v>
+      </c>
       <c r="P485" s="5" t="s">
         <v>128</v>
       </c>
@@ -44752,14 +44765,20 @@
       </c>
       <c r="B486" s="5"/>
       <c r="C486" s="5" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="D486" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E486" s="5"/>
-      <c r="F486" s="5"/>
-      <c r="G486" s="5"/>
+      <c r="E486" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F486" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G486" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="H486" s="5" t="s">
         <v>77</v>
       </c>
@@ -44772,11 +44791,11 @@
       </c>
       <c r="L486" s="6">
         <f t="shared" si="16"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M486" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="N486" s="5"/>
       <c r="O486" s="5" t="s">
@@ -55793,11 +55812,11 @@
       </c>
       <c r="E2" s="8">
         <f>COUNTA(Roster!D2:D715)</f>
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F2" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E2/COUNTA(Roster!A2:A715))</f>
-        <v>0.59105960264900659</v>
+        <v>0.5927152317880795</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -55815,11 +55834,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!E2:E715)</f>
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E3/COUNTA(Roster!A2:A715))</f>
-        <v>0.52152317880794707</v>
+        <v>0.52483443708609268</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -55837,11 +55856,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!F2:F715)</f>
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E4/COUNTA(Roster!A2:A715))</f>
-        <v>0.50496688741721851</v>
+        <v>0.50827814569536423</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -55859,11 +55878,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!G2:G715)</f>
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E5/COUNTA(Roster!A2:A715))</f>
-        <v>0.62748344370860931</v>
+        <v>0.62913907284768211</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -55903,11 +55922,11 @@
       </c>
       <c r="E7" s="8">
         <f>COUNTA(Roster!I2:I715)</f>
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F7" s="9">
         <f>IF(COUNTA(Roster!A2:A715)=0,0,E7/COUNTA(Roster!A2:A715))</f>
-        <v>0.58609271523178808</v>
+        <v>0.58774834437086088</v>
       </c>
     </row>
   </sheetData>
@@ -55950,11 +55969,11 @@
       </c>
       <c r="C2" s="6">
         <f>COUNTIF(Roster!$I$2:$I$715,A2)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" s="10">
         <f t="shared" ref="D2:D13" si="0">IF(SUM($C$2:$C$13)=0,0,C2/SUM($C$2:$C$13))</f>
-        <v>7.909604519774012E-2</v>
+        <v>8.1690140845070425E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -55970,7 +55989,7 @@
       </c>
       <c r="D3" s="10">
         <f t="shared" si="0"/>
-        <v>0.13559322033898305</v>
+        <v>0.13521126760563379</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -55986,7 +56005,7 @@
       </c>
       <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>9.03954802259887E-2</v>
+        <v>9.014084507042254E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -56002,7 +56021,7 @@
       </c>
       <c r="D5" s="10">
         <f t="shared" si="0"/>
-        <v>5.6497175141242938E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -56018,7 +56037,7 @@
       </c>
       <c r="D6" s="10">
         <f t="shared" si="0"/>
-        <v>0.11864406779661017</v>
+        <v>0.11830985915492957</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -56034,7 +56053,7 @@
       </c>
       <c r="D7" s="10">
         <f t="shared" si="0"/>
-        <v>0.12994350282485875</v>
+        <v>0.12957746478873239</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -56050,7 +56069,7 @@
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.11016949152542373</v>
+        <v>0.10985915492957747</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -56066,7 +56085,7 @@
       </c>
       <c r="D9" s="10">
         <f t="shared" si="0"/>
-        <v>0.10734463276836158</v>
+        <v>0.10704225352112676</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -56082,7 +56101,7 @@
       </c>
       <c r="D10" s="10">
         <f t="shared" si="0"/>
-        <v>6.4971751412429377E-2</v>
+        <v>6.4788732394366194E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -56098,7 +56117,7 @@
       </c>
       <c r="D11" s="10">
         <f t="shared" si="0"/>
-        <v>3.3898305084745763E-2</v>
+        <v>3.3802816901408447E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -56114,7 +56133,7 @@
       </c>
       <c r="D12" s="10">
         <f t="shared" si="0"/>
-        <v>3.954802259887006E-2</v>
+        <v>3.9436619718309862E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -56130,7 +56149,7 @@
       </c>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>3.3898305084745763E-2</v>
+        <v>3.3802816901408447E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -56139,7 +56158,7 @@
       </c>
       <c r="C14" s="11">
         <f>SUM(C2:C13)</f>
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -56278,7 +56297,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!M2:M715,"Yes")</f>
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1720</v>
@@ -56290,7 +56309,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.5266666666666666</v>
+        <v>1.54</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1720</v>
@@ -56302,7 +56321,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!L2:L715),0)</f>
-        <v>3.6258278145695364</v>
+        <v>3.6374172185430464</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1720</v>

</xml_diff>

<commit_message>
Fixed errors with Arc names
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C65C7E-99B6-4CF1-9706-F41574ACA41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1C082B-5989-48EF-8F4B-1DEA216C92B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15664,9 +15664,11 @@
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="5"/>
+        <v>43</v>
+      </c>
+      <c r="D5" s="5">
+        <v>25.5</v>
+      </c>
       <c r="E5" s="5" t="s">
         <v>76</v>
       </c>
@@ -15872,7 +15874,9 @@
       <c r="C8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="5"/>
+      <c r="D8" s="5">
+        <v>28.5</v>
+      </c>
       <c r="E8" s="5" t="s">
         <v>44</v>
       </c>
@@ -19645,7 +19649,9 @@
       <c r="C67" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D67" s="5"/>
+      <c r="D67" s="5">
+        <v>26.3</v>
+      </c>
       <c r="E67" s="5" t="s">
         <v>44</v>
       </c>
@@ -19895,7 +19901,9 @@
       <c r="C71" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D71" s="5"/>
+      <c r="D71" s="5">
+        <v>10.6</v>
+      </c>
       <c r="E71" s="5" t="s">
         <v>44</v>
       </c>
@@ -20955,7 +20963,7 @@
       </c>
       <c r="B89" s="5"/>
       <c r="C89" s="5" t="s">
-        <v>128</v>
+        <v>318</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>319</v>
@@ -22487,7 +22495,9 @@
       <c r="C113" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D113" s="5"/>
+      <c r="D113" s="5">
+        <v>21.6</v>
+      </c>
       <c r="E113" s="5" t="s">
         <v>44</v>
       </c>
@@ -25471,7 +25481,7 @@
       </c>
       <c r="B159" s="5"/>
       <c r="C159" s="5" t="s">
-        <v>128</v>
+        <v>318</v>
       </c>
       <c r="D159" s="5" t="s">
         <v>1912</v>
@@ -27771,7 +27781,7 @@
       </c>
       <c r="B197" s="5"/>
       <c r="C197" s="5" t="s">
-        <v>128</v>
+        <v>318</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>319</v>
@@ -56004,7 +56014,7 @@
         <v/>
       </c>
       <c r="N704" s="6" t="str">
-        <f t="shared" ref="N704:N767" si="25">IF(A704="","",IF(AND(M704=6,UPPER(S704)&lt;&gt;"Y",C704&lt;&gt;""),"Yes","No"))</f>
+        <f t="shared" ref="N704:N713" si="25">IF(A704="","",IF(AND(M704=6,UPPER(S704)&lt;&gt;"Y",C704&lt;&gt;""),"Yes","No"))</f>
         <v/>
       </c>
       <c r="O704" s="5"/>
@@ -56323,7 +56333,7 @@
       <sortCondition ref="A1:A713"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="C23:D23 D2:D202 N2:Q713 D204:D713">
+  <conditionalFormatting sqref="D2:D202 N2:Q713 C23:D23 D204:D713">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -56349,7 +56359,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>C2:D22 C203 C24:D202 C204:D713</xm:sqref>
+          <xm:sqref>C204:D713 C203 C24:D202 C2:D22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>

</xml_diff>

<commit_message>
Updated Edict and Licit
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1C082B-5989-48EF-8F4B-1DEA216C92B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFF058A-B9D9-4D62-8F09-655B0FE6E4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10759" uniqueCount="2017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10765" uniqueCount="2018">
   <si>
     <t>Parahumandle – design workbook</t>
   </si>
@@ -6103,6 +6103,9 @@
   </si>
   <si>
     <t>Capable of flight and can turn himself and his gear into a living projectile, unable to change course.</t>
+  </si>
+  <si>
+    <t>x.1</t>
   </si>
 </sst>
 </file>
@@ -25245,7 +25248,7 @@
       </c>
       <c r="B155" s="5"/>
       <c r="C155" s="5" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
@@ -25307,9 +25310,11 @@
       </c>
       <c r="B156" s="5"/>
       <c r="C156" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D156" s="5"/>
+        <v>128</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>2017</v>
+      </c>
       <c r="E156" s="5" t="s">
         <v>76</v>
       </c>
@@ -25319,7 +25324,9 @@
       <c r="G156" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="H156" s="5"/>
+      <c r="H156" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="I156" s="5" t="s">
         <v>58</v>
       </c>
@@ -25332,11 +25339,11 @@
       </c>
       <c r="M156" s="6">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N156" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="O156" s="5"/>
       <c r="P156" s="5" t="s">
@@ -34923,15 +34930,23 @@
       </c>
       <c r="B314" s="5"/>
       <c r="C314" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D314" s="5"/>
+        <v>128</v>
+      </c>
+      <c r="D314" s="5" t="s">
+        <v>2017</v>
+      </c>
       <c r="E314" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F314" s="5"/>
-      <c r="G314" s="5"/>
-      <c r="H314" s="5"/>
+      <c r="F314" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G314" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H314" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="I314" s="5" t="s">
         <v>58</v>
       </c>
@@ -34944,11 +34959,11 @@
       </c>
       <c r="M314" s="6">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N314" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="O314" s="5"/>
       <c r="P314" s="5" t="s">
@@ -56359,7 +56374,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>C204:D713 C203 C24:D202 C2:D22</xm:sqref>
+          <xm:sqref>C24:D202 C203 C2:D22 C204:D713</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000001000000}">
           <x14:formula1>
@@ -56489,11 +56504,11 @@
       </c>
       <c r="E3" s="8">
         <f>COUNTA(Roster!F2:F713)</f>
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F3" s="9">
         <f>IF(COUNTA(Roster!A2:A713)=0,0,E3/COUNTA(Roster!A2:A713))</f>
-        <v>0.58471760797342198</v>
+        <v>0.58637873754152825</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -56511,11 +56526,11 @@
       </c>
       <c r="E4" s="8">
         <f>COUNTA(Roster!G2:G713)</f>
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F4" s="9">
         <f>IF(COUNTA(Roster!A2:A713)=0,0,E4/COUNTA(Roster!A2:A713))</f>
-        <v>0.56810631229235875</v>
+        <v>0.56976744186046513</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -56533,11 +56548,11 @@
       </c>
       <c r="E5" s="8">
         <f>COUNTA(Roster!H2:H713)</f>
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F5" s="9">
         <f>IF(COUNTA(Roster!A2:A713)=0,0,E5/COUNTA(Roster!A2:A713))</f>
-        <v>0.66279069767441856</v>
+        <v>0.66611295681063121</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -56952,7 +56967,7 @@
       </c>
       <c r="B11" s="8">
         <f>COUNTIF(Roster!N2:N713,"Yes")</f>
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>1713</v>
@@ -56964,7 +56979,7 @@
       </c>
       <c r="B12" s="9">
         <f>IF(B5=0,0,B11/B5)</f>
-        <v>1.8333333333333333</v>
+        <v>1.8466666666666667</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>1713</v>
@@ -56976,7 +56991,7 @@
       </c>
       <c r="B13" s="13">
         <f>IFERROR(AVERAGE(Roster!M2:M713),0)</f>
-        <v>3.8787375415282392</v>
+        <v>3.8853820598006643</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>1713</v>

</xml_diff>

<commit_message>
Fixed Number Man's status
</commit_message>
<xml_diff>
--- a/data/parahumandle_design.xlsx
+++ b/data/parahumandle_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Worm Wordle clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427CE6EC-3310-4197-A30A-632E443D55AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D3005B0-48DD-47BB-BB60-98CC5A36DFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48876,7 +48876,7 @@
         <v>46</v>
       </c>
       <c r="H541" s="5" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="I541" s="5" t="s">
         <v>312</v>

</xml_diff>